<commit_message>
Update Swiggy logic: dynamic orders, multi-header ads, and positive adjustments
</commit_message>
<xml_diff>
--- a/template_files/recon_template.xlsx
+++ b/template_files/recon_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Varun\Desktop\Backup AutoRecons\Zomato Auto recons\template_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08EB1343-EF87-43C5-9E5E-EDD285E9D7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D3F36B9-AD7B-4352-BCBD-F60DF4D8F41B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="POS" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">Cashflow!$A$1:$I$38</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Cashflow!$A$1:$I$39</definedName>
     <definedName name="Summary">#REF!</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="79">
   <si>
     <t>Details</t>
   </si>
@@ -265,6 +265,12 @@
   </si>
   <si>
     <t>Swiggy Discrepancies - July 2026</t>
+  </si>
+  <si>
+    <t>Previous week Adjustments</t>
+  </si>
+  <si>
+    <t>Previous Week Adjustments</t>
   </si>
 </sst>
 </file>
@@ -1026,13 +1032,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>175325</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>914017</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>91440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1124,13 +1130,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>175260</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>106680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>913952</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3292,7 +3298,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z1001"/>
+  <dimension ref="A1:Z1002"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.109375" style="97" customWidth="1"/>
@@ -4084,10 +4090,10 @@
       </c>
       <c r="J31" s="4"/>
     </row>
-    <row r="32" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" s="101" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6"/>
       <c r="B32" s="6" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="C32" s="31">
         <v>0</v>
@@ -4108,94 +4114,119 @@
         <f>SUM(C32:G32)</f>
         <v>0</v>
       </c>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-    </row>
-    <row r="33" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J32" s="102"/>
+    </row>
+    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6"/>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C33" s="31">
+        <v>0</v>
+      </c>
+      <c r="D33" s="31">
+        <v>0</v>
+      </c>
+      <c r="E33" s="31">
+        <v>0</v>
+      </c>
+      <c r="F33" s="31">
+        <v>0</v>
+      </c>
+      <c r="G33" s="31">
+        <v>0</v>
+      </c>
+      <c r="H33" s="31">
+        <f>SUM(C33:G33)</f>
+        <v>0</v>
+      </c>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+    </row>
+    <row r="34" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="6"/>
+      <c r="B34" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="88">
-        <v>0</v>
-      </c>
-      <c r="D33" s="88">
-        <v>0</v>
-      </c>
-      <c r="E33" s="88">
-        <v>0</v>
-      </c>
-      <c r="F33" s="88">
-        <v>0</v>
-      </c>
-      <c r="G33" s="88">
-        <v>0</v>
-      </c>
-      <c r="H33" s="59">
-        <f>SUM(C33:G33)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="105">
+      <c r="C34" s="88">
+        <v>0</v>
+      </c>
+      <c r="D34" s="88">
+        <v>0</v>
+      </c>
+      <c r="E34" s="88">
+        <v>0</v>
+      </c>
+      <c r="F34" s="88">
+        <v>0</v>
+      </c>
+      <c r="G34" s="88">
+        <v>0</v>
+      </c>
+      <c r="H34" s="59">
+        <f>SUM(C34:G34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="105">
         <v>8</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B35" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C34" s="89">
-        <f>C30-C31-C32-C33</f>
-        <v>0</v>
-      </c>
-      <c r="D34" s="64">
-        <f>D30-D31-D32-D33</f>
-        <v>0</v>
-      </c>
-      <c r="E34" s="64">
-        <f>E30-E31-E32-E33</f>
-        <v>0</v>
-      </c>
-      <c r="F34" s="64">
-        <f>F30-F31-F32-F33</f>
-        <v>0</v>
-      </c>
-      <c r="G34" s="64">
-        <f>G30-G31-G32-G33</f>
-        <v>0</v>
-      </c>
-      <c r="H34" s="89">
-        <f>SUM(C34:G34)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C35" s="90"/>
-      <c r="D35" s="66"/>
-      <c r="E35" s="91"/>
-      <c r="F35" s="91"/>
-      <c r="G35" s="91"/>
+      <c r="C35" s="89">
+        <f>C30-C31-C33-C34-C32</f>
+        <v>0</v>
+      </c>
+      <c r="D35" s="89">
+        <f t="shared" ref="D35:G35" si="3">D30-D31-D33-D34-D32</f>
+        <v>0</v>
+      </c>
+      <c r="E35" s="89">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="F35" s="89">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G35" s="89">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="H35" s="89">
+        <f>SUM(C35:G35)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="92"/>
-      <c r="B36" s="92" t="s">
+      <c r="C36" s="90"/>
+      <c r="D36" s="66"/>
+      <c r="E36" s="91"/>
+      <c r="F36" s="91"/>
+      <c r="G36" s="91"/>
+    </row>
+    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="92"/>
+      <c r="B37" s="92" t="s">
         <v>49</v>
       </c>
-      <c r="C36" s="93"/>
-      <c r="D36" s="94"/>
-      <c r="E36" s="93"/>
-      <c r="F36" s="93"/>
-      <c r="G36" s="93"/>
-      <c r="K36" s="4"/>
-    </row>
-    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="112"/>
-      <c r="C37" s="107"/>
-      <c r="D37" s="107"/>
-      <c r="E37" s="107"/>
-      <c r="F37" s="107"/>
-      <c r="G37" s="29"/>
-    </row>
-    <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="C37" s="93"/>
+      <c r="D37" s="94"/>
+      <c r="E37" s="93"/>
+      <c r="F37" s="93"/>
+      <c r="G37" s="93"/>
+      <c r="K37" s="4"/>
+    </row>
+    <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="112"/>
+      <c r="C38" s="107"/>
+      <c r="D38" s="107"/>
+      <c r="E38" s="107"/>
+      <c r="F38" s="107"/>
+      <c r="G38" s="29"/>
+    </row>
     <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -5159,11 +5190,12 @@
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="1001" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1002" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B38:F38"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0" footer="0"/>
@@ -6605,7 +6637,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z1001"/>
+  <dimension ref="A1:Z1002"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" style="20" customWidth="1"/>
@@ -6935,28 +6967,28 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8" s="101" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="C19" s="62">
-        <f>Cashflow!C33</f>
-        <v>0</v>
-      </c>
-      <c r="D19" s="62">
-        <f>Cashflow!D33</f>
-        <v>0</v>
-      </c>
-      <c r="E19" s="62">
-        <f>Cashflow!E33</f>
-        <v>0</v>
-      </c>
-      <c r="F19" s="62">
-        <f>Cashflow!F33</f>
-        <v>0</v>
-      </c>
-      <c r="G19" s="62">
-        <f>Cashflow!G33</f>
+        <v>78</v>
+      </c>
+      <c r="C19" s="31">
+        <f>Cashflow!C32</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="31">
+        <f>Cashflow!D32</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="31">
+        <f>Cashflow!E32</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="31">
+        <f>Cashflow!F32</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="31">
+        <f>Cashflow!G32</f>
         <v>0</v>
       </c>
       <c r="H19" s="31">
@@ -6965,55 +6997,81 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="63" t="s">
+      <c r="B20" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" s="62">
+        <f>Cashflow!C34</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="62">
+        <f>Cashflow!D34</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="62">
+        <f>Cashflow!E34</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="62">
+        <f>Cashflow!F34</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="62">
+        <f>Cashflow!G34</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="31">
+        <f>SUM(C20:G20)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="64">
-        <f t="shared" ref="C20:H20" si="1">C17-C19-C18</f>
-        <v>0</v>
-      </c>
-      <c r="D20" s="64">
+      <c r="C21" s="64">
+        <f t="shared" ref="C21:F21" si="1">C17-C20-C18-C19</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E20" s="64">
+      <c r="E21" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F20" s="64">
+      <c r="F21" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G20" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H20" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="52"/>
+      <c r="G21" s="64">
+        <f>G17-G20-G18-G19</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="64">
+        <f>H17-H20-H18-H19</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="22" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="65" t="s">
+      <c r="B22" s="52"/>
+    </row>
+    <row r="23" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="65" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="115"/>
-      <c r="C23" s="107"/>
-      <c r="D23" s="107"/>
-      <c r="E23" s="107"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-    </row>
-    <row r="25" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="52"/>
-    </row>
+    <row r="24" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="115"/>
+      <c r="C24" s="107"/>
+      <c r="D24" s="107"/>
+      <c r="E24" s="107"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19"/>
+    </row>
+    <row r="26" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="27" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="52"/>
     </row>
@@ -7608,22 +7666,24 @@
     <row r="224" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B224" s="52"/>
     </row>
-    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="225" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B225" s="52"/>
+    </row>
+    <row r="226" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="227" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="228" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="229" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="230" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="231" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="232" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="233" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="234" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="235" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="236" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="237" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="238" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="239" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="240" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -8385,11 +8445,12 @@
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="1001" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1002" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B24:E24"/>
     <mergeCell ref="B2:H2"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0" footer="0"/>

</xml_diff>